<commit_message>
Relist 1597 due to box damage, update price and name
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -112,6 +112,12 @@
     <font>
       <name val="微軟正黑體"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <strike val="0"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="14">
@@ -250,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -386,6 +392,15 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2603,25 +2618,25 @@
       <c r="E87" s="44" t="n"/>
     </row>
     <row r="88" ht="15.3" customHeight="1">
-      <c r="A88" s="27" t="inlineStr">
+      <c r="A88" s="48" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B88" s="27" t="inlineStr">
+      <c r="B88" s="48" t="inlineStr">
         <is>
           <t>#1597</t>
         </is>
       </c>
-      <c r="C88" s="27" t="inlineStr">
-        <is>
-          <t>The Mind Flayer (超大盒 奪心魔)</t>
-        </is>
-      </c>
-      <c r="D88" s="35" t="n">
-        <v>500</v>
-      </c>
-      <c r="E88" s="36" t="n"/>
+      <c r="C88" s="48" t="inlineStr">
+        <is>
+          <t>The Mind Flayer (超大盒 奪心魔) (輕微盒損)</t>
+        </is>
+      </c>
+      <c r="D88" s="49" t="n">
+        <v>400</v>
+      </c>
+      <c r="E88" s="50" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2807,12 +2822,11 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>#1547 Demogorgon (Scoops Ahoy 冰淇淋魔王)
-#1597 The Mind Flayer (超大盒 奪心魔)</t>
+          <t>#1547 Demogorgon (Scoops Ahoy 冰淇淋魔王)</t>
         </is>
       </c>
       <c r="C9" s="31" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D9" s="32" t="n"/>
       <c r="E9" s="32" t="n"/>

</xml_diff>

<commit_message>
Update Excel 1595 and 1596 to regular size and price 700
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -2473,7 +2473,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>🦖 大型/場景組</t>
+          <t>📦 常規小盒</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
@@ -2483,18 +2483,18 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Vecna (6吋 豪華大型款)</t>
+          <t>Vecna</t>
         </is>
       </c>
       <c r="D81" s="43" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="E81" s="44" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>🦖 大型/場景組</t>
+          <t>📦 常規小盒</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Demogorgon (6吋 豪華大型款)</t>
+          <t>Demogorgon</t>
         </is>
       </c>
       <c r="D82" s="43" t="n">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="E82" s="44" t="n"/>
     </row>

</xml_diff>

<commit_message>
Relist 675 and update sales record
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -117,6 +117,10 @@
       <name val="微軟正黑體"/>
       <strike val="0"/>
       <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -256,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -402,6 +406,7 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -767,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="25" customWidth="1" style="2" min="1" max="1"/>
@@ -2637,6 +2642,27 @@
         <v>400</v>
       </c>
       <c r="E88" s="50" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="51" t="inlineStr">
+        <is>
+          <t>👑 殿堂與限定熱門款</t>
+        </is>
+      </c>
+      <c r="B89" s="51" t="inlineStr">
+        <is>
+          <t>#675</t>
+        </is>
+      </c>
+      <c r="C89" s="51" t="inlineStr">
+        <is>
+          <t>Steve (SDCC 限定)</t>
+        </is>
+      </c>
+      <c r="D89" s="51" t="n">
+        <v>700</v>
+      </c>
+      <c r="E89" s="51" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2746,14 +2772,13 @@
       <c r="B5" s="8" t="inlineStr">
         <is>
           <t>#674 Robin
-#675 Steve (SDCC 限定)
 #552 Max
 #421 Eleven (Eggos 限定)
 Alexie</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>2200</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="6" ht="57.6" customHeight="1">

</xml_diff>

<commit_message>
Fix formatting for 1597 and 675 in inventory list
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -260,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -407,6 +407,12 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -2623,46 +2629,46 @@
       <c r="E87" s="44" t="n"/>
     </row>
     <row r="88" ht="15.3" customHeight="1">
-      <c r="A88" s="48" t="inlineStr">
+      <c r="A88" s="3" t="inlineStr">
         <is>
           <t>🦖 大型/場景組</t>
         </is>
       </c>
-      <c r="B88" s="48" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>#1597</t>
         </is>
       </c>
-      <c r="C88" s="48" t="inlineStr">
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>The Mind Flayer (超大盒 奪心魔) (輕微盒損)</t>
         </is>
       </c>
-      <c r="D88" s="49" t="n">
+      <c r="D88" s="33" t="n">
         <v>400</v>
       </c>
-      <c r="E88" s="50" t="n"/>
+      <c r="E88" s="34" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="51" t="inlineStr">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>👑 殿堂與限定熱門款</t>
         </is>
       </c>
-      <c r="B89" s="51" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>#675</t>
         </is>
       </c>
-      <c r="C89" s="51" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>Steve (SDCC 限定)</t>
         </is>
       </c>
-      <c r="D89" s="51" t="n">
+      <c r="D89" s="52" t="n">
         <v>750</v>
       </c>
-      <c r="E89" s="51" t="n"/>
+      <c r="E89" s="53" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Change regular small boxes to pink fill in Excel
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -124,7 +124,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -221,6 +221,12 @@
         <bgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+        <bgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -278,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -478,6 +484,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1094,25 +1115,25 @@
       <c r="E11" s="58" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B12" s="59" t="inlineStr">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B12" s="70" t="inlineStr">
         <is>
           <t>#425</t>
         </is>
       </c>
-      <c r="C12" s="59" t="inlineStr">
+      <c r="C12" s="70" t="inlineStr">
         <is>
           <t>Lucas (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D12" s="60" t="n">
+      <c r="D12" s="71" t="n">
         <v>850</v>
       </c>
-      <c r="E12" s="61" t="n"/>
+      <c r="E12" s="72" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="57" t="inlineStr">
@@ -1137,216 +1158,216 @@
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B14" s="59" t="inlineStr">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="inlineStr">
         <is>
           <t>#427</t>
         </is>
       </c>
-      <c r="C14" s="59" t="inlineStr">
+      <c r="C14" s="70" t="inlineStr">
         <is>
           <t>Barb (第一季經典) (2016購入已絕版)</t>
         </is>
       </c>
-      <c r="D14" s="60" t="n">
+      <c r="D14" s="71" t="n">
         <v>700</v>
       </c>
-      <c r="E14" s="61" t="n"/>
+      <c r="E14" s="72" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B15" s="59" t="inlineStr">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B15" s="70" t="inlineStr">
         <is>
           <t>#428</t>
         </is>
       </c>
-      <c r="C15" s="59" t="inlineStr">
+      <c r="C15" s="70" t="inlineStr">
         <is>
           <t>Demogorgon (魔王開口款)</t>
         </is>
       </c>
-      <c r="D15" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E15" s="61" t="n"/>
+      <c r="D15" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E15" s="72" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B16" s="59" t="inlineStr">
+      <c r="A16" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="inlineStr">
         <is>
           <t>#436</t>
         </is>
       </c>
-      <c r="C16" s="59" t="inlineStr">
+      <c r="C16" s="70" t="inlineStr">
         <is>
           <t>Joyce (第一季聖誕燈泡)</t>
         </is>
       </c>
-      <c r="D16" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E16" s="61" t="n"/>
+      <c r="D16" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E16" s="72" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B17" s="59" t="inlineStr">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B17" s="70" t="inlineStr">
         <is>
           <t>#512</t>
         </is>
       </c>
-      <c r="C17" s="59" t="inlineStr">
+      <c r="C17" s="70" t="inlineStr">
         <is>
           <t>Hopper (警長常規款)</t>
         </is>
       </c>
-      <c r="D17" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E17" s="61" t="n"/>
+      <c r="D17" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E17" s="72" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B18" s="59" t="inlineStr">
+      <c r="A18" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B18" s="70" t="inlineStr">
         <is>
           <t>#513</t>
         </is>
       </c>
-      <c r="C18" s="59" t="inlineStr">
+      <c r="C18" s="70" t="inlineStr">
         <is>
           <t>Jonathan (第一季照相機)</t>
         </is>
       </c>
-      <c r="D18" s="60" t="n">
+      <c r="D18" s="71" t="n">
         <v>750</v>
       </c>
-      <c r="E18" s="61" t="n"/>
+      <c r="E18" s="72" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="A19" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B19" s="70" t="inlineStr">
         <is>
           <t>#514</t>
         </is>
       </c>
-      <c r="C19" s="59" t="inlineStr">
+      <c r="C19" s="70" t="inlineStr">
         <is>
           <t>Nancy (第一季拿槍款)</t>
         </is>
       </c>
-      <c r="D19" s="60" t="n">
+      <c r="D19" s="71" t="n">
         <v>750</v>
       </c>
-      <c r="E19" s="61" t="n"/>
+      <c r="E19" s="72" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="A20" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B20" s="70" t="inlineStr">
         <is>
           <t>#515</t>
         </is>
       </c>
-      <c r="C20" s="59" t="inlineStr">
+      <c r="C20" s="70" t="inlineStr">
         <is>
           <t>Brenner (布倫納博士)</t>
         </is>
       </c>
-      <c r="D20" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E20" s="61" t="n"/>
+      <c r="D20" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E20" s="72" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B21" s="59" t="inlineStr">
+      <c r="A21" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B21" s="70" t="inlineStr">
         <is>
           <t>#545</t>
         </is>
       </c>
-      <c r="C21" s="59" t="inlineStr">
+      <c r="C21" s="70" t="inlineStr">
         <is>
           <t>Eleven (實驗室病人服)</t>
         </is>
       </c>
-      <c r="D21" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E21" s="61" t="n"/>
+      <c r="D21" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E21" s="72" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B22" s="59" t="inlineStr">
+      <c r="A22" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B22" s="70" t="inlineStr">
         <is>
           <t>#550</t>
         </is>
       </c>
-      <c r="C22" s="59" t="inlineStr">
+      <c r="C22" s="70" t="inlineStr">
         <is>
           <t>Joyce (磁鐵版)</t>
         </is>
       </c>
-      <c r="D22" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E22" s="61" t="n"/>
+      <c r="D22" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E22" s="72" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="A23" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B23" s="70" t="inlineStr">
         <is>
           <t>#572</t>
         </is>
       </c>
-      <c r="C23" s="59" t="inlineStr">
+      <c r="C23" s="70" t="inlineStr">
         <is>
           <t>Eleven (BoxLunch 限定 吊帶褲)</t>
         </is>
       </c>
-      <c r="D23" s="60" t="inlineStr">
+      <c r="D23" s="71" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="E23" s="61" t="n"/>
+      <c r="E23" s="72" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="57" t="inlineStr">
@@ -1370,109 +1391,109 @@
       <c r="E24" s="58" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B25" s="59" t="inlineStr">
+      <c r="A25" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B25" s="70" t="inlineStr">
         <is>
           <t>#637</t>
         </is>
       </c>
-      <c r="C25" s="59" t="inlineStr">
+      <c r="C25" s="70" t="inlineStr">
         <is>
           <t>Eleven (Elevated 升空施法)</t>
         </is>
       </c>
-      <c r="D25" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E25" s="61" t="n"/>
+      <c r="D25" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E25" s="72" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B26" s="59" t="inlineStr">
+      <c r="A26" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B26" s="70" t="inlineStr">
         <is>
           <t>#640</t>
         </is>
       </c>
-      <c r="C26" s="59" t="inlineStr">
+      <c r="C26" s="70" t="inlineStr">
         <is>
           <t>Billy (比利經典款)</t>
         </is>
       </c>
-      <c r="D26" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E26" s="61" t="n"/>
+      <c r="D26" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E26" s="72" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B27" s="59" t="inlineStr">
+      <c r="A27" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B27" s="70" t="inlineStr">
         <is>
           <t>#643</t>
         </is>
       </c>
-      <c r="C27" s="59" t="inlineStr">
+      <c r="C27" s="70" t="inlineStr">
         <is>
           <t>Vampire Bob (吸血鬼鮑伯)</t>
         </is>
       </c>
-      <c r="D27" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E27" s="61" t="n"/>
+      <c r="D27" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E27" s="72" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B28" s="59" t="inlineStr">
+      <c r="A28" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B28" s="70" t="inlineStr">
         <is>
           <t>#674</t>
         </is>
       </c>
-      <c r="C28" s="59" t="inlineStr">
+      <c r="C28" s="70" t="inlineStr">
         <is>
           <t>Robin (冰淇淋制服款)</t>
         </is>
       </c>
-      <c r="D28" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E28" s="61" t="n"/>
+      <c r="D28" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E28" s="72" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="62" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B29" s="62" t="inlineStr">
+      <c r="A29" s="73" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B29" s="73" t="inlineStr">
         <is>
           <t>#675</t>
         </is>
       </c>
-      <c r="C29" s="62" t="inlineStr">
+      <c r="C29" s="73" t="inlineStr">
         <is>
           <t>Steve (SDCC 限定)</t>
         </is>
       </c>
-      <c r="D29" s="63" t="n">
+      <c r="D29" s="74" t="n">
         <v>750</v>
       </c>
-      <c r="E29" s="61" t="n"/>
+      <c r="E29" s="72" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="57" t="inlineStr">
@@ -1496,25 +1517,25 @@
       <c r="E30" s="58" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B31" s="59" t="inlineStr">
+      <c r="A31" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B31" s="70" t="inlineStr">
         <is>
           <t>#720</t>
         </is>
       </c>
-      <c r="C31" s="59" t="inlineStr">
+      <c r="C31" s="70" t="inlineStr">
         <is>
           <t>Hopper (約會襯衫款)</t>
         </is>
       </c>
-      <c r="D31" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E31" s="61" t="n"/>
+      <c r="D31" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E31" s="72" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="57" t="inlineStr">
@@ -1538,132 +1559,132 @@
       <c r="E32" s="58" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B33" s="59" t="inlineStr">
+      <c r="A33" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B33" s="70" t="inlineStr">
         <is>
           <t>#803</t>
         </is>
       </c>
-      <c r="C33" s="59" t="inlineStr">
+      <c r="C33" s="70" t="inlineStr">
         <is>
           <t>Steve (拿聖代冰淇淋款)</t>
         </is>
       </c>
-      <c r="D33" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E33" s="61" t="n"/>
+      <c r="D33" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E33" s="72" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B34" s="59" t="inlineStr">
+      <c r="A34" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B34" s="70" t="inlineStr">
         <is>
           <t>#804</t>
         </is>
       </c>
-      <c r="C34" s="59" t="inlineStr">
+      <c r="C34" s="70" t="inlineStr">
         <is>
           <t>Dustin (Walmart 限定 夏令營帽子)</t>
         </is>
       </c>
-      <c r="D34" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E34" s="61" t="n"/>
+      <c r="D34" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E34" s="72" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B35" s="59" t="inlineStr">
+      <c r="A35" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B35" s="70" t="inlineStr">
         <is>
           <t>#807</t>
         </is>
       </c>
-      <c r="C35" s="59" t="inlineStr">
+      <c r="C35" s="70" t="inlineStr">
         <is>
           <t>Lucas (S3 商場造型)</t>
         </is>
       </c>
-      <c r="D35" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E35" s="61" t="n"/>
+      <c r="D35" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E35" s="72" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B36" s="59" t="inlineStr">
+      <c r="A36" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B36" s="70" t="inlineStr">
         <is>
           <t>#808</t>
         </is>
       </c>
-      <c r="C36" s="59" t="inlineStr">
+      <c r="C36" s="70" t="inlineStr">
         <is>
           <t>Erica (經典款)</t>
         </is>
       </c>
-      <c r="D36" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E36" s="61" t="n"/>
+      <c r="D36" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E36" s="72" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B37" s="59" t="inlineStr">
+      <c r="A37" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B37" s="70" t="inlineStr">
         <is>
           <t>#826</t>
         </is>
       </c>
-      <c r="C37" s="59" t="inlineStr">
+      <c r="C37" s="70" t="inlineStr">
         <is>
           <t>Battle Eleven (商場大戰眼罩款)</t>
         </is>
       </c>
-      <c r="D37" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E37" s="61" t="n"/>
+      <c r="D37" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E37" s="72" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B38" s="59" t="inlineStr">
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B38" s="70" t="inlineStr">
         <is>
           <t>#827</t>
         </is>
       </c>
-      <c r="C38" s="59" t="inlineStr">
+      <c r="C38" s="70" t="inlineStr">
         <is>
           <t>Eleven (紅色外套)</t>
         </is>
       </c>
-      <c r="D38" s="60" t="inlineStr">
+      <c r="D38" s="71" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="E38" s="61" t="n"/>
+      <c r="E38" s="72" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="57" t="inlineStr">
@@ -1687,67 +1708,67 @@
       <c r="E39" s="58" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B40" s="59" t="inlineStr">
+      <c r="A40" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B40" s="70" t="inlineStr">
         <is>
           <t>#843</t>
         </is>
       </c>
-      <c r="C40" s="59" t="inlineStr">
+      <c r="C40" s="70" t="inlineStr">
         <is>
           <t>Eleven (黑色幾何圖騰洋裝)</t>
         </is>
       </c>
-      <c r="D40" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E40" s="61" t="n"/>
+      <c r="D40" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E40" s="72" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B41" s="59" t="inlineStr">
+      <c r="A41" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B41" s="70" t="inlineStr">
         <is>
           <t>#922</t>
         </is>
       </c>
-      <c r="C41" s="59" t="inlineStr">
+      <c r="C41" s="70" t="inlineStr">
         <is>
           <t>Robin (拿白板款)</t>
         </is>
       </c>
-      <c r="D41" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E41" s="61" t="n"/>
+      <c r="D41" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E41" s="72" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B42" s="59" t="inlineStr">
+      <c r="A42" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B42" s="70" t="inlineStr">
         <is>
           <t>#1241</t>
         </is>
       </c>
-      <c r="C42" s="59" t="inlineStr">
+      <c r="C42" s="70" t="inlineStr">
         <is>
           <t>Lucas (S4 籃球隊服)</t>
         </is>
       </c>
-      <c r="D42" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E42" s="61" t="n"/>
+      <c r="D42" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E42" s="72" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="57" t="inlineStr">
@@ -1771,25 +1792,25 @@
       <c r="E43" s="58" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B44" s="59" t="inlineStr">
+      <c r="A44" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B44" s="70" t="inlineStr">
         <is>
           <t>#1301</t>
         </is>
       </c>
-      <c r="C44" s="59" t="inlineStr">
+      <c r="C44" s="70" t="inlineStr">
         <is>
           <t>Erica (S4 戰鬥裝備)</t>
         </is>
       </c>
-      <c r="D44" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E44" s="61" t="n"/>
+      <c r="D44" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E44" s="72" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="57" t="inlineStr">
@@ -1834,67 +1855,67 @@
       <c r="E46" s="58" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B47" s="59" t="inlineStr">
+      <c r="A47" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B47" s="70" t="inlineStr">
         <is>
           <t>#1457</t>
         </is>
       </c>
-      <c r="C47" s="59" t="inlineStr">
+      <c r="C47" s="70" t="inlineStr">
         <is>
           <t>Eleven (S4 流鼻血戰鬥款)</t>
         </is>
       </c>
-      <c r="D47" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E47" s="61" t="n"/>
+      <c r="D47" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E47" s="72" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B48" s="59" t="inlineStr">
+      <c r="A48" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B48" s="70" t="inlineStr">
         <is>
           <t>#1459</t>
         </is>
       </c>
-      <c r="C48" s="59" t="inlineStr">
+      <c r="C48" s="70" t="inlineStr">
         <is>
           <t>Jonathan (S4 經典款)</t>
         </is>
       </c>
-      <c r="D48" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E48" s="61" t="n"/>
+      <c r="D48" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E48" s="72" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B49" s="59" t="inlineStr">
+      <c r="A49" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B49" s="70" t="inlineStr">
         <is>
           <t>#1461</t>
         </is>
       </c>
-      <c r="C49" s="59" t="inlineStr">
+      <c r="C49" s="70" t="inlineStr">
         <is>
           <t>Robin (貝雷帽款式)</t>
         </is>
       </c>
-      <c r="D49" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E49" s="61" t="n"/>
+      <c r="D49" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E49" s="72" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="57" t="inlineStr">
@@ -1918,151 +1939,151 @@
       <c r="E50" s="58" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B51" s="59" t="inlineStr">
+      <c r="A51" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B51" s="70" t="inlineStr">
         <is>
           <t>#1463</t>
         </is>
       </c>
-      <c r="C51" s="59" t="inlineStr">
+      <c r="C51" s="70" t="inlineStr">
         <is>
           <t>Dustin (地獄火盾牌長矛)</t>
         </is>
       </c>
-      <c r="D51" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E51" s="61" t="n"/>
+      <c r="D51" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E51" s="72" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B52" s="59" t="inlineStr">
+      <c r="A52" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B52" s="70" t="inlineStr">
         <is>
           <t>#1538</t>
         </is>
       </c>
-      <c r="C52" s="59" t="inlineStr">
+      <c r="C52" s="70" t="inlineStr">
         <is>
           <t>Chrissy (啦啦隊長)</t>
         </is>
       </c>
-      <c r="D52" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E52" s="61" t="n"/>
+      <c r="D52" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E52" s="72" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B53" s="59" t="inlineStr">
+      <c r="A53" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B53" s="70" t="inlineStr">
         <is>
           <t>#1540</t>
         </is>
       </c>
-      <c r="C53" s="59" t="inlineStr">
+      <c r="C53" s="70" t="inlineStr">
         <is>
           <t>Vecna (S4 常規款)</t>
         </is>
       </c>
-      <c r="D53" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E53" s="61" t="n"/>
+      <c r="D53" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E53" s="72" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B54" s="59" t="inlineStr">
+      <c r="A54" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B54" s="70" t="inlineStr">
         <is>
           <t>#1542</t>
         </is>
       </c>
-      <c r="C54" s="59" t="inlineStr">
+      <c r="C54" s="70" t="inlineStr">
         <is>
           <t>Steve (顛倒世界拿手電筒)</t>
         </is>
       </c>
-      <c r="D54" s="60" t="n">
+      <c r="D54" s="71" t="n">
         <v>800</v>
       </c>
-      <c r="E54" s="61" t="n"/>
+      <c r="E54" s="72" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B55" s="59" t="inlineStr">
+      <c r="A55" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B55" s="70" t="inlineStr">
         <is>
           <t>#1543</t>
         </is>
       </c>
-      <c r="C55" s="59" t="inlineStr">
+      <c r="C55" s="70" t="inlineStr">
         <is>
           <t>Murray (火焰噴射器)</t>
         </is>
       </c>
-      <c r="D55" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E55" s="61" t="n"/>
+      <c r="D55" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E55" s="72" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B56" s="59" t="inlineStr">
+      <c r="A56" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B56" s="70" t="inlineStr">
         <is>
           <t>#1545</t>
         </is>
       </c>
-      <c r="C56" s="59" t="inlineStr">
+      <c r="C56" s="70" t="inlineStr">
         <is>
           <t>Steve (Scoops Ahoy 復古包裝)</t>
         </is>
       </c>
-      <c r="D56" s="60" t="n">
+      <c r="D56" s="71" t="n">
         <v>750</v>
       </c>
-      <c r="E56" s="61" t="n"/>
+      <c r="E56" s="72" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B57" s="59" t="inlineStr">
+      <c r="A57" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B57" s="70" t="inlineStr">
         <is>
           <t>#1546</t>
         </is>
       </c>
-      <c r="C57" s="59" t="inlineStr">
+      <c r="C57" s="70" t="inlineStr">
         <is>
           <t>Robin (Scoops Ahoy 復古包裝)</t>
         </is>
       </c>
-      <c r="D57" s="60" t="n">
+      <c r="D57" s="71" t="n">
         <v>750</v>
       </c>
-      <c r="E57" s="61" t="n"/>
+      <c r="E57" s="72" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="57" t="inlineStr">
@@ -2086,67 +2107,67 @@
       <c r="E58" s="58" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B59" s="59" t="inlineStr">
+      <c r="A59" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B59" s="70" t="inlineStr">
         <is>
           <t>#1559</t>
         </is>
       </c>
-      <c r="C59" s="59" t="inlineStr">
+      <c r="C59" s="70" t="inlineStr">
         <is>
           <t>001 Vaporizing (2024 SDCC 消散版) (有2隻)</t>
         </is>
       </c>
-      <c r="D59" s="60" t="n">
+      <c r="D59" s="71" t="n">
         <v>700</v>
       </c>
-      <c r="E59" s="61" t="n"/>
+      <c r="E59" s="72" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="62" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B60" s="62" t="inlineStr">
+      <c r="A60" s="73" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B60" s="73" t="inlineStr">
         <is>
           <t>#1595</t>
         </is>
       </c>
-      <c r="C60" s="62" t="inlineStr">
+      <c r="C60" s="73" t="inlineStr">
         <is>
           <t>Vecna</t>
         </is>
       </c>
-      <c r="D60" s="63" t="n">
+      <c r="D60" s="74" t="n">
         <v>700</v>
       </c>
-      <c r="E60" s="61" t="n"/>
+      <c r="E60" s="72" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="62" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B61" s="62" t="inlineStr">
+      <c r="A61" s="73" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B61" s="73" t="inlineStr">
         <is>
           <t>#1596</t>
         </is>
       </c>
-      <c r="C61" s="62" t="inlineStr">
+      <c r="C61" s="73" t="inlineStr">
         <is>
           <t>Demogorgon</t>
         </is>
       </c>
-      <c r="D61" s="63" t="n">
+      <c r="D61" s="74" t="n">
         <v>700</v>
       </c>
-      <c r="E61" s="61" t="n"/>
+      <c r="E61" s="72" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="57" t="inlineStr">
@@ -2170,130 +2191,130 @@
       <c r="E62" s="58" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B63" s="59" t="inlineStr">
+      <c r="A63" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B63" s="70" t="inlineStr">
         <is>
           <t>#1780</t>
         </is>
       </c>
-      <c r="C63" s="59" t="inlineStr">
+      <c r="C63" s="70" t="inlineStr">
         <is>
           <t>Eleven (Season 5)</t>
         </is>
       </c>
-      <c r="D63" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E63" s="61" t="n"/>
+      <c r="D63" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E63" s="72" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B64" s="59" t="inlineStr">
+      <c r="A64" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B64" s="70" t="inlineStr">
         <is>
           <t>#1781</t>
         </is>
       </c>
-      <c r="C64" s="59" t="inlineStr">
+      <c r="C64" s="70" t="inlineStr">
         <is>
           <t>Dustin Henderson (Season 5)</t>
         </is>
       </c>
-      <c r="D64" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E64" s="61" t="n"/>
+      <c r="D64" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E64" s="72" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B65" s="59" t="inlineStr">
+      <c r="A65" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B65" s="70" t="inlineStr">
         <is>
           <t>#1782</t>
         </is>
       </c>
-      <c r="C65" s="59" t="inlineStr">
+      <c r="C65" s="70" t="inlineStr">
         <is>
           <t>Holly Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D65" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E65" s="61" t="n"/>
+      <c r="D65" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E65" s="72" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B66" s="59" t="inlineStr">
+      <c r="A66" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B66" s="70" t="inlineStr">
         <is>
           <t>#1783</t>
         </is>
       </c>
-      <c r="C66" s="59" t="inlineStr">
+      <c r="C66" s="70" t="inlineStr">
         <is>
           <t>Mike Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D66" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E66" s="61" t="n"/>
+      <c r="D66" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E66" s="72" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B67" s="59" t="inlineStr">
+      <c r="A67" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B67" s="70" t="inlineStr">
         <is>
           <t>#1784</t>
         </is>
       </c>
-      <c r="C67" s="59" t="inlineStr">
+      <c r="C67" s="70" t="inlineStr">
         <is>
           <t>Jim Hopper (Season 5)</t>
         </is>
       </c>
-      <c r="D67" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E67" s="61" t="n"/>
+      <c r="D67" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E67" s="72" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B68" s="59" t="inlineStr">
+      <c r="A68" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B68" s="70" t="inlineStr">
         <is>
           <t>#1785</t>
         </is>
       </c>
-      <c r="C68" s="59" t="inlineStr">
+      <c r="C68" s="70" t="inlineStr">
         <is>
           <t>Lucas Sinclair (Season 5)</t>
         </is>
       </c>
-      <c r="D68" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E68" s="61" t="n"/>
+      <c r="D68" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E68" s="72" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="57" t="inlineStr">
@@ -2359,151 +2380,151 @@
       <c r="E71" s="58" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B72" s="59" t="inlineStr">
+      <c r="A72" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B72" s="70" t="inlineStr">
         <is>
           <t>#1798</t>
         </is>
       </c>
-      <c r="C72" s="59" t="inlineStr">
+      <c r="C72" s="70" t="inlineStr">
         <is>
           <t>Lucas Sinclair (S5 WSQK 特別款)</t>
         </is>
       </c>
-      <c r="D72" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E72" s="61" t="n"/>
+      <c r="D72" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E72" s="72" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B73" s="59" t="inlineStr">
+      <c r="A73" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B73" s="70" t="inlineStr">
         <is>
           <t>#1802</t>
         </is>
       </c>
-      <c r="C73" s="59" t="inlineStr">
+      <c r="C73" s="70" t="inlineStr">
         <is>
           <t>Nancy Wheeler (Season 5)</t>
         </is>
       </c>
-      <c r="D73" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E73" s="61" t="n"/>
+      <c r="D73" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E73" s="72" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B74" s="59" t="inlineStr">
+      <c r="A74" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B74" s="70" t="inlineStr">
         <is>
           <t>#1805</t>
         </is>
       </c>
-      <c r="C74" s="59" t="inlineStr">
+      <c r="C74" s="70" t="inlineStr">
         <is>
           <t>Max Mayfield (Season 5)</t>
         </is>
       </c>
-      <c r="D74" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E74" s="61" t="n"/>
+      <c r="D74" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E74" s="72" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B75" s="59" t="inlineStr">
+      <c r="A75" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B75" s="70" t="inlineStr">
         <is>
           <t>#1807</t>
         </is>
       </c>
-      <c r="C75" s="59" t="inlineStr">
+      <c r="C75" s="70" t="inlineStr">
         <is>
           <t>Eleven (Season 5)</t>
         </is>
       </c>
-      <c r="D75" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E75" s="61" t="n"/>
+      <c r="D75" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E75" s="72" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B76" s="59" t="inlineStr">
+      <c r="A76" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B76" s="70" t="inlineStr">
         <is>
           <t>#1808</t>
         </is>
       </c>
-      <c r="C76" s="59" t="inlineStr">
+      <c r="C76" s="70" t="inlineStr">
         <is>
           <t>Mr. Whatsit (Season 5)</t>
         </is>
       </c>
-      <c r="D76" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E76" s="61" t="n"/>
+      <c r="D76" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E76" s="72" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B77" s="59" t="inlineStr">
+      <c r="A77" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B77" s="70" t="inlineStr">
         <is>
           <t>#1810</t>
         </is>
       </c>
-      <c r="C77" s="59" t="inlineStr">
+      <c r="C77" s="70" t="inlineStr">
         <is>
           <t>Holly The Heroic (S5 英雄霍莉)</t>
         </is>
       </c>
-      <c r="D77" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E77" s="61" t="n"/>
+      <c r="D77" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E77" s="72" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="59" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B78" s="59" t="inlineStr">
+      <c r="A78" s="70" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B78" s="70" t="inlineStr">
         <is>
           <t>#1831</t>
         </is>
       </c>
-      <c r="C78" s="59" t="inlineStr">
+      <c r="C78" s="70" t="inlineStr">
         <is>
           <t>Demogorgon (S5 最新魔王款)</t>
         </is>
       </c>
-      <c r="D78" s="60" t="n">
-        <v>500</v>
-      </c>
-      <c r="E78" s="61" t="n"/>
+      <c r="D78" s="71" t="n">
+        <v>500</v>
+      </c>
+      <c r="E78" s="72" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="64" t="inlineStr">

</xml_diff>

<commit_message>
Sell 675, 674, 436, 1463 for 2200
</commit_message>
<xml_diff>
--- a/剩餘庫存清單-Scott專用格式.xlsx
+++ b/剩餘庫存清單-Scott專用格式.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="新細明體"/>
       <family val="2"/>
@@ -120,8 +120,18 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <strike val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微軟正黑體"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -194,8 +204,26 @@
         <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCC0DA"/>
+        <bgColor rgb="00CCC0DA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -248,11 +276,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -339,6 +381,18 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -976,25 +1030,25 @@
       <c r="E12" s="25" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>#436</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Joyce (第一季聖誕燈泡)</t>
         </is>
       </c>
-      <c r="D13" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E13" s="25" t="n"/>
+      <c r="D13" s="31" t="n">
+        <v>500</v>
+      </c>
+      <c r="E13" s="32" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
@@ -1272,46 +1326,46 @@
       <c r="E26" s="25" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t>#674</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>Robin (冰淇淋制服款)</t>
         </is>
       </c>
-      <c r="D27" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E27" s="25" t="n"/>
+      <c r="D27" s="31" t="n">
+        <v>500</v>
+      </c>
+      <c r="E27" s="32" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="26" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B28" s="26" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
         <is>
           <t>#675</t>
         </is>
       </c>
-      <c r="C28" s="26" t="inlineStr">
+      <c r="C28" s="31" t="inlineStr">
         <is>
           <t>Steve (SDCC 限定)</t>
         </is>
       </c>
-      <c r="D28" s="27" t="n">
+      <c r="D28" s="31" t="n">
         <v>750</v>
       </c>
-      <c r="E28" s="25" t="n"/>
+      <c r="E28" s="32" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
@@ -1925,25 +1979,25 @@
       <c r="E57" s="19" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="23" t="inlineStr">
-        <is>
-          <t>📦 常規小盒</t>
-        </is>
-      </c>
-      <c r="B58" s="23" t="inlineStr">
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>📦 常規小盒</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
         <is>
           <t>#1463</t>
         </is>
       </c>
-      <c r="C58" s="23" t="inlineStr">
+      <c r="C58" s="31" t="inlineStr">
         <is>
           <t>Dustin (地獄火盾牌長矛)</t>
         </is>
       </c>
-      <c r="D58" s="24" t="n">
-        <v>500</v>
-      </c>
-      <c r="E58" s="25" t="n"/>
+      <c r="D58" s="31" t="n">
+        <v>500</v>
+      </c>
+      <c r="E58" s="32" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="23" t="inlineStr">
@@ -2607,7 +2661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" style="2" min="1" max="1"/>
@@ -2823,6 +2877,24 @@
         <v>500</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="inlineStr">
+        <is>
+          <t>#436 Joyce (第一季聖誕燈泡)
+#674 Robin (冰淇淋制服款)
+#675 Steve (SDCC 限定)
+#1463 Dustin (地獄火盾牌長矛)</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="n">
+        <v>2200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>